<commit_message>
Cap nhat trang thai da dang cho 13 bai blog SEO
</commit_message>
<xml_diff>
--- a/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
+++ b/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Đã viết xong - sẵn sàng đăng</t>
+          <t>Đã đăng</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Them 3 bai blog SEO: Phan Thiet, Tay Ninh, Nha Trang
</commit_message>
<xml_diff>
--- a/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
+++ b/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1079,6 +1079,117 @@
       <c r="G16" s="4" t="inlineStr">
         <is>
           <t>thue-xe-carnival-di-cong-tac-tinh.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Phan Thiết Tự Túc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>thuê xe Carnival đi Phan Thiết</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-phan-thiet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Tây Ninh, Núi Bà Đen Trong Ngày</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>thuê xe Carnival đi Tây Ninh Núi Bà Đen</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-tay-ninh.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Nha Trang Đường Dài</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>thuê xe Carnival đi Nha Trang</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-nha-trang.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Them Google Analytics, 19 trang SEO moi va internal link toan site
- Gan the GA4 (G-4YGYG2JRJF) vao toan bo 61 trang
- 16 bai blog moi (tuyen mien Tay, Moc Bai, Long Hai, city tour, phu phi...)
  kem FAQPage + BreadcrumbList schema
- 3 trang landing: Quan 1, Go Vap, tong hop tuyen mien Tay
- Khoi "Bai viet lien quan" cho moi bai blog va "Cam nang" cho trang dich vu
- Cap nhat blog index, sitemap, lich dang bai, danh sach 100 tu khoa
- Sua gia sai "450.000d/ngay" trong bai 1 xe hay 2 xe

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
+++ b/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1190,6 +1190,598 @@
       <c r="G19" t="inlineStr">
         <is>
           <t>kinh-nghiem-thue-xe-di-nha-trang.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gia Đình Đông Người: Nên Thuê 1 Xe Carnival Hay 2 Xe Nhỏ?</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nên thuê 1 xe hay 2 xe cho gia đình đông người</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>So sánh</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>So sánh</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nen-thue-1-xe-carnival-hay-2-xe-nho.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Về Quê Dịp Tết Nguyên Đán</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>thuê xe về quê Tết</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-ve-que-tet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Thuê Xe Carnival Đón Đối Tác, Khách VIP Tại Sân Bay</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>thuê xe đón đối tác VIP sân bay</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Dịch vụ đặc biệt</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>thue-xe-carnival-don-doi-tac-vip-san-bay.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe 7 Chỗ Đi Bến Tre Từ TP.HCM: Lịch Trình 1 Ngày Xứ Dừa</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ đi Bến Tre</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-ben-tre.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Thuê Xe Carnival Đi Cửa Khẩu Mộc Bài: Giá, Lộ Trình Và Lưu Ý Qua Biên</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>thuê xe đi cửa khẩu Mộc Bài</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>thue-xe-carnival-di-cua-khau-moc-bai.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Rạch Giá, Nối Chuyến Tàu Ra Phú Quốc</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>thuê xe đi Rạch Giá</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-rach-gia.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Bạc Liêu – Cà Mau Về Đất Mũi</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>thuê xe đi Cà Mau Bạc Liêu</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-bac-lieu-ca-mau.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Châu Đốc Viếng Bà Chúa Xứ Núi Sam</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>thuê xe đi Châu Đốc</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-chau-doc-an-giang.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Thuê Xe Carnival City Tour Sài Gòn 1 Ngày: Lịch Trình Cho Gia Đình Và Khách Nước Ngoài</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>thuê xe city tour Sài Gòn</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>thue-xe-carnival-city-tour-sai-gon.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Thuê Xe Có Tài Xế Đưa Đón Ông Bà, Người Lớn Tuổi Đi Khám Bệnh Tại TP.HCM</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>thuê xe đưa người già đi khám bệnh</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Dịch vụ đặc biệt</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>thue-xe-carnival-dua-don-nguoi-gia-di-kham-benh.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Cách Tính Phí Phát Sinh Khi Thuê Xe Có Tài Xế: Vượt Giờ, Vượt Km, Cầu Đường</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>phí phát sinh thuê xe có tài xế</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>So sánh</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bảng giá</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>cach-tinh-phi-phat-sinh-thue-xe-co-tai-xe.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>So Sánh Kia Carnival Với Innova, Fortuner, Xpander Khi Thuê Xe 7 Chỗ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>nên thuê Carnival hay Innova Fortuner</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>So sánh</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>So sánh</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>so-sanh-kia-carnival-voi-cac-dong-xe-7-cho.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Thuê Xe Carnival Theo Giờ Tại TP.HCM: 6 Tình Huống Nên Dùng Để Tiết Kiệm</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ theo giờ TP.HCM</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Hướng dẫn</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>khi-nao-nen-thue-xe-carnival-theo-gio.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe 7 Chỗ Đi Long Hải – Hồ Tràm Cuối Tuần</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ đi Long Hải Hồ Tràm</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-long-hai-ho-tram.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Sóc Trăng: Chùa Khmer, Bánh Pía Và Lễ Hội Oóc Om Bóc</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ đi Sóc Trăng</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-soc-trang.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Thuê Xe Carnival Đi Vĩnh Long: Cù Lao An Bình, Làng Gốm Mang Thít</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ đi Vĩnh Long</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Đã đăng</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-di-vinh-long.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Them 10 bai ve tinh va anchor text chua tu khoa cho internal link
- 10 bai moi: diem don san bay TSN, san bay Long Thanh, tu lai Vung Tau,
  tu lai Da Lat, Cu Chi, Can Gio, Binh Duong, dua don nhan vien,
  Bao Loc, checklist thue xe lan dau
- Anchor dan ve trang chinh xoay vong 3-4 bien the chua tu khoa
- Moi bai blog co them link ve trang chu
- Cap nhat blog index, sitemap, lich dang bai

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
+++ b/Lich_Dang_Bai_SEO_ThueXeCarnival.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1782,6 +1782,376 @@
       <c r="G35" t="inlineStr">
         <is>
           <t>kinh-nghiem-thue-xe-di-vinh-long.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Điểm Đón Xe Sân Bay Tân Sơn Nhất Ở Đâu? Hướng Dẫn Ga T1, T2, T3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>điểm đón xe sân bay Tân Sơn Nhất</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Hướng dẫn</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>diem-don-xe-san-bay-tan-son-nhat.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Thuê Xe 7 Chỗ Đi Sân Bay Long Thành: Quãng Đường, Thời Gian Và Lưu Ý</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>thuê xe đi sân bay Long Thành</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Hướng dẫn</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>thue-xe-di-san-bay-long-thanh.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Thuê Xe Tự Lái Đi Vũng Tàu: Chi Phí, Lộ Trình Và Kinh Nghiệm Giữ Cọc</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>thuê xe tự lái đi Vũng Tàu</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm thuê xe</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>thue-xe-tu-lai-di-vung-tau.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Kinh Nghiệm Tự Lái Xe 7 Chỗ Đi Đà Lạt: Đèo Bảo Lộc, Điểm Nghỉ Và Định Mức Km</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>kinh nghiệm tự lái xe đi Đà Lạt</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm thuê xe</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-tu-lai-xe-di-da-lat.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Thuê Xe 7 Chỗ Đi Địa Đạo Củ Chi Trong Ngày: Lịch Trình Và Chi Phí</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>thuê xe đi địa đạo Củ Chi</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>thue-xe-di-dia-dao-cu-chi.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Thuê Xe 7 Chỗ Đi Cần Giờ Trong Ngày: Rừng Sác, Đảo Khỉ Và Hải Sản</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>thuê xe đi Cần Giờ</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>thue-xe-di-can-gio.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Thuê Xe 7 Chỗ Đi Bình Dương: Đại Nam, Khu Công Nghiệp Và Công Tác</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ đi Bình Dương</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>thue-xe-7-cho-di-binh-duong.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Thuê Xe Đưa Đón Nhân Viên, Chuyên Gia Hằng Ngày: Theo Tháng Hay Theo Ngày?</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>thuê xe đưa đón nhân viên hằng ngày</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>So sánh</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>thue-xe-dua-don-nhan-vien-hang-ngay.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Thuê Xe 7 Chỗ Đi Bảo Lộc: Đồi Chè, Thác Đambri Và Điểm Nghỉ Trên Đường Đà Lạt</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>thuê xe đi Bảo Lộc</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Mua ngay</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Kinh nghiệm du lịch</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>thue-xe-di-bao-loc.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Lần Đầu Thuê Xe 7 Chỗ Có Tài Xế Tại TP.HCM: Checklist 10 Điều Cần Hỏi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>thuê xe 7 chỗ có tài xế lần đầu</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Tìm hiểu</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Hướng dẫn</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Đã viết - chưa đăng</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>kinh-nghiem-thue-xe-7-cho-co-tai-xe-lan-dau.html</t>
         </is>
       </c>
     </row>

</xml_diff>